<commit_message>
dirty the indexes to check tool resilience
</commit_message>
<xml_diff>
--- a/mapping.xlsx
+++ b/mapping.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8719d062a8aedec1/Documents/Projects/bates-pager/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8719d062a8aedec1/Documents/Projects/bates-mapper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_F25DC773A252ABDACC1048DA291F6FA05BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAAC652F-781F-4A51-9559-A52DBFD2C942}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_F25DC773A252ABDACC1048DA291F6FA05BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CC24A40-8C08-43E3-AE2C-E3E77F393BDB}"/>
   <bookViews>
     <workbookView xWindow="15645" yWindow="4665" windowWidth="26715" windowHeight="14175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -167,6 +167,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -432,230 +436,230 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="B2:D22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="D3">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="C3">
+      <c r="D4">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C5" t="s">
         <v>7</v>
       </c>
-      <c r="C4">
+      <c r="D5">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="C5">
+      <c r="D6">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C7" t="s">
         <v>7</v>
       </c>
-      <c r="C6">
+      <c r="D7">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C8" t="s">
         <v>11</v>
       </c>
-      <c r="C7">
+      <c r="D8">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C9" t="s">
         <v>11</v>
       </c>
-      <c r="C8">
+      <c r="D9">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C10" t="s">
         <v>14</v>
       </c>
-      <c r="C9">
+      <c r="D10">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
         <v>15</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C11" t="s">
         <v>14</v>
       </c>
-      <c r="C10">
+      <c r="D11">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C12" t="s">
         <v>14</v>
       </c>
-      <c r="C11">
+      <c r="D12">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
         <v>17</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C13" t="s">
         <v>18</v>
       </c>
-      <c r="C12">
+      <c r="D13">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C14" t="s">
         <v>18</v>
       </c>
-      <c r="C13">
+      <c r="D14">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
         <v>20</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C15" t="s">
         <v>21</v>
       </c>
-      <c r="C14">
+      <c r="D15">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
         <v>22</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C16" t="s">
         <v>21</v>
       </c>
-      <c r="C15">
+      <c r="D16">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
         <v>23</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C17" t="s">
         <v>24</v>
       </c>
-      <c r="C16">
+      <c r="D17">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
         <v>25</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C18" t="s">
         <v>24</v>
       </c>
-      <c r="C17">
+      <c r="D18">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
         <v>26</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C19" t="s">
         <v>26</v>
       </c>
-      <c r="C18">
+      <c r="D19">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
         <v>27</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C20" t="s">
         <v>27</v>
       </c>
-      <c r="C19">
+      <c r="D20">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>